<commit_message>
Update Week 7 AMS weekly data and processed ads files
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Tonor/business_report_week7.xlsx
+++ b/data/ams_weekly_data/Tonor/business_report_week7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\ams_weekly_data\Tonor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2055C576-F62A-4006-A8BE-ECF7A31E7988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D90DFFE-65E9-4531-8E38-95EB0104C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="112">
   <si>
     <t>(Parent) ASIN</t>
   </si>
@@ -93,405 +93,72 @@
     <t>Total Order Items - B2B</t>
   </si>
   <si>
-    <t>0.23%</t>
-  </si>
-  <si>
-    <t>0.51%</t>
-  </si>
-  <si>
-    <t>0.50%</t>
-  </si>
-  <si>
-    <t>12.50%</t>
-  </si>
-  <si>
-    <t>100.00%</t>
-  </si>
-  <si>
-    <t>0.00%</t>
-  </si>
-  <si>
-    <t>₹0.00</t>
-  </si>
-  <si>
-    <t>0.38%</t>
-  </si>
-  <si>
-    <t>0.52%</t>
-  </si>
-  <si>
-    <t>0.30%</t>
-  </si>
-  <si>
-    <t>0.61%</t>
-  </si>
-  <si>
-    <t>0.36%</t>
-  </si>
-  <si>
-    <t>0.31%</t>
-  </si>
-  <si>
-    <t>0.90%</t>
-  </si>
-  <si>
-    <t>0.45%</t>
-  </si>
-  <si>
-    <t>0.12%</t>
-  </si>
-  <si>
-    <t>0.13%</t>
-  </si>
-  <si>
-    <t>0.22%</t>
-  </si>
-  <si>
-    <t>0.76%</t>
-  </si>
-  <si>
-    <t>8.33%</t>
-  </si>
-  <si>
-    <t>0.04%</t>
-  </si>
-  <si>
-    <t>0.06%</t>
-  </si>
-  <si>
-    <t>0.01%</t>
-  </si>
-  <si>
-    <t>0.18%</t>
-  </si>
-  <si>
-    <t>0.32%</t>
-  </si>
-  <si>
-    <t>0.17%</t>
-  </si>
-  <si>
-    <t>1.52%</t>
-  </si>
-  <si>
-    <t>0.85%</t>
-  </si>
-  <si>
-    <t>0.19%</t>
-  </si>
-  <si>
-    <t>0.44%</t>
-  </si>
-  <si>
-    <t>0.24%</t>
-  </si>
-  <si>
-    <t>0.21%</t>
-  </si>
-  <si>
-    <t>0.69%</t>
-  </si>
-  <si>
-    <t>0.10%</t>
-  </si>
-  <si>
-    <t>0.15%</t>
-  </si>
-  <si>
-    <t>0.41%</t>
-  </si>
-  <si>
-    <t>0.40%</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>0.02%</t>
-  </si>
-  <si>
-    <t>0.03%</t>
-  </si>
-  <si>
-    <t>2.92%</t>
-  </si>
-  <si>
-    <t>0.11%</t>
-  </si>
-  <si>
-    <t>0.27%</t>
-  </si>
-  <si>
-    <t>0.09%</t>
-  </si>
-  <si>
-    <t>648</t>
-  </si>
-  <si>
-    <t>0.64%</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>88</t>
-  </si>
-  <si>
-    <t>1.90%</t>
-  </si>
-  <si>
-    <t>1.42%</t>
-  </si>
-  <si>
-    <t>0.86%</t>
-  </si>
-  <si>
-    <t>201</t>
-  </si>
-  <si>
-    <t>0.82%</t>
-  </si>
-  <si>
-    <t>0.28%</t>
-  </si>
-  <si>
-    <t>0.55%</t>
-  </si>
-  <si>
-    <t>286</t>
-  </si>
-  <si>
-    <t>0.67%</t>
-  </si>
-  <si>
-    <t>11.11%</t>
-  </si>
-  <si>
-    <t>157</t>
-  </si>
-  <si>
-    <t>140</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>1.85%</t>
-  </si>
-  <si>
-    <t>0.68%</t>
-  </si>
-  <si>
-    <t>0.54%</t>
-  </si>
-  <si>
-    <t>0.58%</t>
-  </si>
-  <si>
-    <t>0.42%</t>
-  </si>
-  <si>
-    <t>6.25%</t>
-  </si>
-  <si>
-    <t>0.14%</t>
-  </si>
-  <si>
-    <t>88.89%</t>
-  </si>
-  <si>
     <t>B08CVP2HXP</t>
   </si>
   <si>
     <t>TONOR USB Microphone, Condenser Computer PC Mic with Tripod Stand, Metal,Pop Filter, Shock Mount for Gaming,Streaming,Podcasting,YouTube, Voice Over,Skype, Twitch,Compatible with Laptop Desktop, TC30</t>
   </si>
   <si>
-    <t>463</t>
-  </si>
-  <si>
-    <t>7.14%</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>₹13,495.00</t>
-  </si>
-  <si>
-    <t>105</t>
-  </si>
-  <si>
-    <t>178</t>
-  </si>
-  <si>
-    <t>0.91%</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
     <t>B07WLWN2ZT</t>
   </si>
   <si>
     <t>TONOR USB Gaming Microphone, Computer Condenser PC Mic with Tripod Stand &amp; Pop for Streaming, Podcasting, Vocal Recording, Compatible with iMac PC Laptop Desktop Windows Computer, TC-777</t>
   </si>
   <si>
-    <t>446</t>
-  </si>
-  <si>
-    <t>589</t>
-  </si>
-  <si>
-    <t>585</t>
-  </si>
-  <si>
-    <t>278</t>
-  </si>
-  <si>
-    <t>1,009</t>
-  </si>
-  <si>
     <t>B0BRKFP94K</t>
   </si>
   <si>
     <t>TONOR TD510 Dynamic Microphone, USB/XLR PC Microphone for Podcast, Recording, Live Streaming &amp; Gaming, XLR Cardioid Studio Mic Music Voice-Over with Quick Mute, Headphone Output, Volume Control</t>
   </si>
   <si>
-    <t>328</t>
-  </si>
-  <si>
-    <t>489</t>
-  </si>
-  <si>
-    <t>66</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>5.56%</t>
-  </si>
-  <si>
-    <t>1.67%</t>
-  </si>
-  <si>
     <t>B07GVGMW59</t>
   </si>
   <si>
     <t>TONOR G11 Conference USB Microphone, Omnidirectional Condenser PC Mic for Video Conference, Recording, Skype, Online Class, Court Reporter, Plug &amp; Play Compatible with Mac OS X Windows PC Computer</t>
   </si>
   <si>
-    <t>444</t>
-  </si>
-  <si>
-    <t>99.74%</t>
-  </si>
-  <si>
-    <t>4.20%</t>
-  </si>
-  <si>
-    <t>15.63%</t>
-  </si>
-  <si>
-    <t>5.39%</t>
-  </si>
-  <si>
     <t>B01ISNU3X4</t>
   </si>
   <si>
     <t>TONOR Dynamic Karaoke Microphone for Singing with 4.5m XLR Cable, Metal Handheld Mic Compatible with Karaoke Machine/Speaker/Amp/Mixer for Karaoke Singing, Speech, Wedding, Stage and Outdoor Activity</t>
   </si>
   <si>
-    <t>1,430</t>
-  </si>
-  <si>
-    <t>12.36%</t>
-  </si>
-  <si>
     <t>B0BYHHSLPC</t>
   </si>
   <si>
     <t>TONOR TC777 Pro Gaming USB Microphone for PC, RGB Condenser Computer Mic with Tripod Stand, Quick Mute, Gain Control, for Gaming, Streaming, Podcasting, Recording, Cardioid Mic Kit for Laptop/PS4/PS5</t>
   </si>
   <si>
-    <t>591</t>
-  </si>
-  <si>
-    <t>913</t>
-  </si>
-  <si>
-    <t>36.04%</t>
-  </si>
-  <si>
     <t>B078WNW4YW</t>
   </si>
   <si>
     <t>TONOR Wireless Microphone Isolation Shield, Mic Sound Absorbing Foam Reflector for Any Condenser Recording Equipment Studio (Black)</t>
   </si>
   <si>
-    <t>193</t>
-  </si>
-  <si>
     <t>B089FVQD3Z</t>
   </si>
   <si>
     <t>Microphone Stand Extension Arm, TONOR Studio Suspension Scissor Boom Arm with Pop Filter, 3/8" to 5/8" Adapter, Mic Clip, Upgraded Heavy Duty Clamp for Blue Yeti Snowball Ice and Other Mics(T30)</t>
   </si>
   <si>
-    <t>34.15%</t>
-  </si>
-  <si>
-    <t>23.36%</t>
-  </si>
-  <si>
     <t>B08NDB5NWP</t>
   </si>
   <si>
     <t>TONOR USB Conference Microphone, 360 Omnidirectional PC Computer Condenser Mic with Mute Button for Online Meeting/Class, Zoom Call, Skype Chatting, Plug &amp; Play (TM20,Red)</t>
   </si>
   <si>
-    <t>51.06%</t>
-  </si>
-  <si>
-    <t>10.21%</t>
-  </si>
-  <si>
     <t>B0BTCXQQ6M</t>
   </si>
   <si>
     <t>TONOR Gaming Mic, USB Microphone for PC Computer, Cardioid Condenser Mic with Adjustable RGB Modes &amp; Brightness, Quick Mute, Gain Control, for Streaming, Podcasting, Recording, PS4/5 Desktop TC310</t>
   </si>
   <si>
-    <t>862</t>
-  </si>
-  <si>
-    <t>9.10%</t>
-  </si>
-  <si>
     <t>B082W4B7SX</t>
   </si>
   <si>
     <t>TONOR Microphone Arm Stand, TONOR Adjustable Suspension Boom Scissor Mic Stand with Pop , 3/8" to 5/8" Adapter, Mic Clip, Upgraded Heavy Duty Clamp for Blue Yeti Nano Snowball Ice and Other Mics(T20)</t>
   </si>
   <si>
-    <t>8.74%</t>
-  </si>
-  <si>
     <t>B08V1JS3NY</t>
   </si>
   <si>
@@ -516,9 +183,6 @@
     <t>TONOR RGB USB Gaming Microphone Kit, Podcast Microphone for PC, One-tap Mute for Streaming, Cardioid Condenser Microphone for PS4/5 Gamer Youtuber, Studio Mic Bundle with Adjustment Arm Stand</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
     <t>B0BRCR2QQ7</t>
   </si>
   <si>
@@ -531,12 +195,6 @@
     <t>TONOR TC310+ RGB Condenser Mic with Boom Arm Quick Mute, RGB Lighting, Pop Filter, Shock Mount,Gaming USB Microphone Set for PC Gain Control for Streaming Podcasting Recording Discord Twitch YouTube</t>
   </si>
   <si>
-    <t>626</t>
-  </si>
-  <si>
-    <t>817</t>
-  </si>
-  <si>
     <t>B0CH9JR3HL</t>
   </si>
   <si>
@@ -553,9 +211,6 @@
   </si>
   <si>
     <t>TONOR TM310 USB Conference Microphone for Laptop, Adjustable Computer PC Mic with Mute Button &amp; LED Indicator for Video Call Meeting, Mic for Desktop Zoom Skype YouTube, Plug-Play for MacOS Windows</t>
-  </si>
-  <si>
-    <t>211</t>
   </si>
   <si>
     <t>ordered_product_sales</t>
@@ -753,9 +408,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1066,10 +724,10 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>176</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>177</v>
+        <v>62</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1111,7 +769,7 @@
         <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>175</v>
+        <v>60</v>
       </c>
       <c r="Q1" t="s">
         <v>13</v>
@@ -1123,7 +781,7 @@
         <v>15</v>
       </c>
       <c r="T1" t="s">
-        <v>174</v>
+        <v>59</v>
       </c>
       <c r="U1" t="s">
         <v>16</v>
@@ -1137,49 +795,49 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>178</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F2" t="s">
-        <v>90</v>
+        <v>20</v>
+      </c>
+      <c r="F2" s="2">
+        <v>463</v>
       </c>
       <c r="G2">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" t="s">
-        <v>63</v>
+      <c r="H2" s="3">
+        <v>1.8E-3</v>
+      </c>
+      <c r="I2" s="3">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="J2" s="2">
+        <v>648</v>
       </c>
       <c r="K2">
         <v>20</v>
       </c>
-      <c r="L2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" t="s">
-        <v>80</v>
-      </c>
-      <c r="O2" t="s">
-        <v>91</v>
+      <c r="L2" s="3">
+        <v>1.9E-3</v>
+      </c>
+      <c r="M2" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="N2" s="3">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="O2" s="3">
+        <v>7.1400000000000005E-2</v>
       </c>
       <c r="P2">
         <v>1</v>
@@ -1187,17 +845,17 @@
       <c r="Q2">
         <v>0</v>
       </c>
-      <c r="R2" t="s">
-        <v>36</v>
-      </c>
-      <c r="S2" t="s">
-        <v>24</v>
+      <c r="R2" s="3">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="S2" s="3">
+        <v>0</v>
       </c>
       <c r="T2" s="1">
         <v>1905.9322033898306</v>
       </c>
-      <c r="U2" t="s">
-        <v>25</v>
+      <c r="U2" s="1">
+        <v>0</v>
       </c>
       <c r="V2">
         <v>1</v>
@@ -1208,49 +866,49 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" t="s">
-        <v>103</v>
+        <v>22</v>
+      </c>
+      <c r="F3" s="2">
+        <v>446</v>
       </c>
       <c r="G3">
         <v>10</v>
       </c>
-      <c r="H3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I3" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" t="s">
-        <v>104</v>
+      <c r="H3" s="3">
+        <v>1.8E-3</v>
+      </c>
+      <c r="I3" s="3">
+        <v>2.0999999999999999E-3</v>
+      </c>
+      <c r="J3" s="2">
+        <v>589</v>
       </c>
       <c r="K3">
         <v>13</v>
       </c>
-      <c r="L3" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s">
-        <v>47</v>
-      </c>
-      <c r="N3" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" t="s">
-        <v>24</v>
+      <c r="L3" s="3">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="M3" s="3">
+        <v>1.9E-3</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3">
+        <v>0</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -1258,17 +916,17 @@
       <c r="Q3">
         <v>0</v>
       </c>
-      <c r="R3" t="s">
-        <v>24</v>
-      </c>
-      <c r="S3" t="s">
-        <v>24</v>
+      <c r="R3" s="3">
+        <v>0</v>
+      </c>
+      <c r="S3" s="3">
+        <v>0</v>
       </c>
       <c r="T3" s="1">
         <v>0</v>
       </c>
-      <c r="U3" t="s">
-        <v>25</v>
+      <c r="U3" s="1">
+        <v>0</v>
       </c>
       <c r="V3">
         <v>0</v>
@@ -1279,49 +937,49 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>183</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F4" t="s">
-        <v>110</v>
+        <v>24</v>
+      </c>
+      <c r="F4" s="2">
+        <v>328</v>
       </c>
       <c r="G4">
         <v>5</v>
       </c>
-      <c r="H4" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" t="s">
-        <v>60</v>
-      </c>
-      <c r="J4" t="s">
-        <v>111</v>
+      <c r="H4" s="3">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="J4" s="2">
+        <v>489</v>
       </c>
       <c r="K4">
         <v>6</v>
       </c>
-      <c r="L4" t="s">
-        <v>86</v>
-      </c>
-      <c r="M4" t="s">
-        <v>62</v>
-      </c>
-      <c r="N4" t="s">
-        <v>49</v>
-      </c>
-      <c r="O4" t="s">
-        <v>24</v>
+      <c r="L4" s="3">
+        <v>1.4E-3</v>
+      </c>
+      <c r="M4" s="3">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="N4" s="3">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="O4" s="3">
+        <v>0</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -1329,17 +987,17 @@
       <c r="Q4">
         <v>0</v>
       </c>
-      <c r="R4" t="s">
-        <v>24</v>
-      </c>
-      <c r="S4" t="s">
-        <v>24</v>
+      <c r="R4" s="3">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3">
+        <v>0</v>
       </c>
       <c r="T4" s="1">
         <v>0</v>
       </c>
-      <c r="U4" t="s">
-        <v>25</v>
+      <c r="U4" s="1">
+        <v>0</v>
       </c>
       <c r="V4">
         <v>0</v>
@@ -1350,49 +1008,49 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" t="s">
-        <v>74</v>
+        <v>26</v>
+      </c>
+      <c r="F5" s="2">
+        <v>286</v>
       </c>
       <c r="G5">
         <v>32</v>
       </c>
-      <c r="H5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J5" t="s">
-        <v>120</v>
+      <c r="H5" s="3">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="I5" s="3">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="J5" s="2">
+        <v>444</v>
       </c>
       <c r="K5">
         <v>52</v>
       </c>
-      <c r="L5" t="s">
-        <v>72</v>
-      </c>
-      <c r="M5" t="s">
-        <v>117</v>
-      </c>
-      <c r="N5" t="s">
-        <v>121</v>
-      </c>
-      <c r="O5" t="s">
-        <v>23</v>
+      <c r="L5" s="3">
+        <v>2.8E-3</v>
+      </c>
+      <c r="M5" s="3">
+        <v>1.67E-2</v>
+      </c>
+      <c r="N5" s="3">
+        <v>0.99739999999999995</v>
+      </c>
+      <c r="O5" s="3">
+        <v>1</v>
       </c>
       <c r="P5">
         <v>12</v>
@@ -1400,17 +1058,17 @@
       <c r="Q5">
         <v>5</v>
       </c>
-      <c r="R5" t="s">
-        <v>122</v>
-      </c>
-      <c r="S5" t="s">
-        <v>123</v>
+      <c r="R5" s="3">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="S5" s="3">
+        <v>0.15629999999999999</v>
       </c>
       <c r="T5" s="1">
         <v>25160.169491525427</v>
       </c>
-      <c r="U5" t="s">
-        <v>93</v>
+      <c r="U5" s="1">
+        <v>13495</v>
       </c>
       <c r="V5">
         <v>12</v>
@@ -1421,49 +1079,49 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="C6" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
-      </c>
-      <c r="F6" t="s">
-        <v>107</v>
+        <v>28</v>
+      </c>
+      <c r="F6" s="4">
+        <v>1009</v>
       </c>
       <c r="G6">
         <v>17</v>
       </c>
-      <c r="H6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>127</v>
+      <c r="H6" s="3">
+        <v>8.6E-3</v>
+      </c>
+      <c r="I6" s="3">
+        <v>7.6E-3</v>
+      </c>
+      <c r="J6" s="4">
+        <v>1430</v>
       </c>
       <c r="K6">
         <v>28</v>
       </c>
-      <c r="L6" t="s">
-        <v>96</v>
-      </c>
-      <c r="M6" t="s">
-        <v>32</v>
-      </c>
-      <c r="N6" t="s">
-        <v>128</v>
-      </c>
-      <c r="O6" t="s">
-        <v>116</v>
+      <c r="L6" s="3">
+        <v>9.1000000000000004E-3</v>
+      </c>
+      <c r="M6" s="3">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="N6" s="3">
+        <v>0.1236</v>
+      </c>
+      <c r="O6" s="3">
+        <v>5.5599999999999997E-2</v>
       </c>
       <c r="P6">
         <v>7</v>
@@ -1471,17 +1129,17 @@
       <c r="Q6">
         <v>0</v>
       </c>
-      <c r="R6" t="s">
-        <v>51</v>
-      </c>
-      <c r="S6" t="s">
-        <v>24</v>
+      <c r="R6" s="3">
+        <v>6.8999999999999999E-3</v>
+      </c>
+      <c r="S6" s="3">
+        <v>0</v>
       </c>
       <c r="T6" s="1">
         <v>10968.644067796611</v>
       </c>
-      <c r="U6" t="s">
-        <v>25</v>
+      <c r="U6" s="1">
+        <v>0</v>
       </c>
       <c r="V6">
         <v>7</v>
@@ -1492,49 +1150,49 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>188</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>189</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>129</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>130</v>
-      </c>
-      <c r="F7" t="s">
-        <v>131</v>
+        <v>30</v>
+      </c>
+      <c r="F7" s="2">
+        <v>591</v>
       </c>
       <c r="G7">
         <v>9</v>
       </c>
-      <c r="H7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" t="s">
-        <v>132</v>
+      <c r="H7" s="3">
+        <v>5.1000000000000004E-3</v>
+      </c>
+      <c r="I7" s="3">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="J7" s="2">
+        <v>913</v>
       </c>
       <c r="K7">
         <v>14</v>
       </c>
-      <c r="L7" t="s">
-        <v>83</v>
-      </c>
-      <c r="M7" t="s">
-        <v>33</v>
-      </c>
-      <c r="N7" t="s">
-        <v>133</v>
-      </c>
-      <c r="O7" t="s">
-        <v>87</v>
+      <c r="L7" s="3">
+        <v>5.7999999999999996E-3</v>
+      </c>
+      <c r="M7" s="3">
+        <v>4.4999999999999997E-3</v>
+      </c>
+      <c r="N7" s="3">
+        <v>0.3604</v>
+      </c>
+      <c r="O7" s="3">
+        <v>0.88890000000000002</v>
       </c>
       <c r="P7">
         <v>5</v>
@@ -1542,17 +1200,17 @@
       <c r="Q7">
         <v>0</v>
       </c>
-      <c r="R7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S7" t="s">
-        <v>24</v>
+      <c r="R7" s="3">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="S7" s="3">
+        <v>0</v>
       </c>
       <c r="T7" s="1">
         <v>8046.610169491526</v>
       </c>
-      <c r="U7" t="s">
-        <v>25</v>
+      <c r="U7" s="1">
+        <v>0</v>
       </c>
       <c r="V7">
         <v>5</v>
@@ -1563,49 +1221,49 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>190</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>191</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>134</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>134</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F8" t="s">
-        <v>136</v>
+        <v>32</v>
+      </c>
+      <c r="F8" s="2">
+        <v>193</v>
       </c>
       <c r="G8">
         <v>5</v>
       </c>
-      <c r="H8" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" t="s">
-        <v>106</v>
+      <c r="H8" s="3">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="I8" s="3">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="J8" s="2">
+        <v>278</v>
       </c>
       <c r="K8">
         <v>7</v>
       </c>
-      <c r="L8" t="s">
-        <v>42</v>
-      </c>
-      <c r="M8" t="s">
-        <v>19</v>
-      </c>
-      <c r="N8" t="s">
-        <v>71</v>
-      </c>
-      <c r="O8" t="s">
-        <v>24</v>
+      <c r="L8" s="3">
+        <v>1.8E-3</v>
+      </c>
+      <c r="M8" s="3">
+        <v>2.3E-3</v>
+      </c>
+      <c r="N8" s="3">
+        <v>8.2000000000000007E-3</v>
+      </c>
+      <c r="O8" s="3">
+        <v>0</v>
       </c>
       <c r="P8">
         <v>1</v>
@@ -1613,17 +1271,17 @@
       <c r="Q8">
         <v>0</v>
       </c>
-      <c r="R8" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" t="s">
-        <v>24</v>
+      <c r="R8" s="3">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="S8" s="3">
+        <v>0</v>
       </c>
       <c r="T8" s="1">
         <v>2202.5423728813562</v>
       </c>
-      <c r="U8" t="s">
-        <v>25</v>
+      <c r="U8" s="1">
+        <v>0</v>
       </c>
       <c r="V8">
         <v>1</v>
@@ -1634,49 +1292,49 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>192</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>193</v>
+        <v>78</v>
       </c>
       <c r="C9" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>138</v>
-      </c>
-      <c r="F9" t="s">
-        <v>112</v>
+        <v>34</v>
+      </c>
+      <c r="F9" s="2">
+        <v>66</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J9" t="s">
-        <v>66</v>
+      <c r="H9" s="3">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="I9" s="3">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="J9" s="2">
+        <v>88</v>
       </c>
       <c r="K9">
         <v>1</v>
       </c>
-      <c r="L9" t="s">
-        <v>40</v>
-      </c>
-      <c r="M9" t="s">
-        <v>58</v>
-      </c>
-      <c r="N9" t="s">
-        <v>139</v>
-      </c>
-      <c r="O9" t="s">
-        <v>24</v>
+      <c r="L9" s="3">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="M9" s="3">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="N9" s="3">
+        <v>0.34150000000000003</v>
+      </c>
+      <c r="O9" s="3">
+        <v>0</v>
       </c>
       <c r="P9">
         <v>1</v>
@@ -1684,17 +1342,17 @@
       <c r="Q9">
         <v>0</v>
       </c>
-      <c r="R9" t="s">
-        <v>45</v>
-      </c>
-      <c r="S9" t="s">
-        <v>24</v>
+      <c r="R9" s="3">
+        <v>1.52E-2</v>
+      </c>
+      <c r="S9" s="3">
+        <v>0</v>
       </c>
       <c r="T9" s="1">
         <v>2456.7796610169494</v>
       </c>
-      <c r="U9" t="s">
-        <v>25</v>
+      <c r="U9" s="1">
+        <v>0</v>
       </c>
       <c r="V9">
         <v>1</v>
@@ -1705,49 +1363,49 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>178</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>179</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
-      </c>
-      <c r="F10" t="s">
-        <v>90</v>
+        <v>20</v>
+      </c>
+      <c r="F10" s="2">
+        <v>463</v>
       </c>
       <c r="G10">
         <v>15</v>
       </c>
-      <c r="H10" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" t="s">
-        <v>75</v>
-      </c>
-      <c r="J10" t="s">
-        <v>63</v>
+      <c r="H10" s="3">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="I10" s="3">
+        <v>6.7000000000000002E-3</v>
+      </c>
+      <c r="J10" s="2">
+        <v>648</v>
       </c>
       <c r="K10">
         <v>20</v>
       </c>
-      <c r="L10" t="s">
-        <v>54</v>
-      </c>
-      <c r="M10" t="s">
-        <v>64</v>
-      </c>
-      <c r="N10" t="s">
-        <v>140</v>
-      </c>
-      <c r="O10" t="s">
-        <v>24</v>
+      <c r="L10" s="3">
+        <v>4.1000000000000003E-3</v>
+      </c>
+      <c r="M10" s="3">
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="N10" s="3">
+        <v>0.2336</v>
+      </c>
+      <c r="O10" s="3">
+        <v>0</v>
       </c>
       <c r="P10">
         <v>1</v>
@@ -1755,17 +1413,17 @@
       <c r="Q10">
         <v>0</v>
       </c>
-      <c r="R10" t="s">
-        <v>36</v>
-      </c>
-      <c r="S10" t="s">
-        <v>24</v>
+      <c r="R10" s="3">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="S10" s="3">
+        <v>0</v>
       </c>
       <c r="T10" s="1">
         <v>1905.9322033898306</v>
       </c>
-      <c r="U10" t="s">
-        <v>25</v>
+      <c r="U10" s="1">
+        <v>0</v>
       </c>
       <c r="V10">
         <v>1</v>
@@ -1776,49 +1434,49 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>194</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
-        <v>195</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>141</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>141</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>142</v>
-      </c>
-      <c r="F11" t="s">
-        <v>94</v>
+        <v>36</v>
+      </c>
+      <c r="F11" s="2">
+        <v>105</v>
       </c>
       <c r="G11">
         <v>8</v>
       </c>
-      <c r="H11" t="s">
-        <v>62</v>
-      </c>
-      <c r="I11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J11" t="s">
-        <v>77</v>
+      <c r="H11" s="3">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="I11" s="3">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="J11" s="2">
+        <v>157</v>
       </c>
       <c r="K11">
         <v>10</v>
       </c>
-      <c r="L11" t="s">
-        <v>52</v>
-      </c>
-      <c r="M11" t="s">
-        <v>43</v>
-      </c>
-      <c r="N11" t="s">
-        <v>143</v>
-      </c>
-      <c r="O11" t="s">
-        <v>22</v>
+      <c r="L11" s="3">
+        <v>1E-3</v>
+      </c>
+      <c r="M11" s="3">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="N11" s="3">
+        <v>0.51060000000000005</v>
+      </c>
+      <c r="O11" s="3">
+        <v>0.125</v>
       </c>
       <c r="P11">
         <v>2</v>
@@ -1826,17 +1484,17 @@
       <c r="Q11">
         <v>0</v>
       </c>
-      <c r="R11" t="s">
-        <v>67</v>
-      </c>
-      <c r="S11" t="s">
-        <v>24</v>
+      <c r="R11" s="3">
+        <v>1.9E-2</v>
+      </c>
+      <c r="S11" s="3">
+        <v>0</v>
       </c>
       <c r="T11" s="1">
         <v>5083.0508474576272</v>
       </c>
-      <c r="U11" t="s">
-        <v>25</v>
+      <c r="U11" s="1">
+        <v>0</v>
       </c>
       <c r="V11">
         <v>1</v>
@@ -1847,49 +1505,49 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>182</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>183</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
-      </c>
-      <c r="F12" t="s">
-        <v>110</v>
+        <v>24</v>
+      </c>
+      <c r="F12" s="2">
+        <v>328</v>
       </c>
       <c r="G12">
         <v>5</v>
       </c>
-      <c r="H12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" t="s">
-        <v>36</v>
-      </c>
-      <c r="J12" t="s">
-        <v>111</v>
+      <c r="H12" s="3">
+        <v>2.8E-3</v>
+      </c>
+      <c r="I12" s="3">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="J12" s="2">
+        <v>489</v>
       </c>
       <c r="K12">
         <v>6</v>
       </c>
-      <c r="L12" t="s">
-        <v>31</v>
-      </c>
-      <c r="M12" t="s">
-        <v>47</v>
-      </c>
-      <c r="N12" t="s">
-        <v>144</v>
-      </c>
-      <c r="O12" t="s">
-        <v>24</v>
+      <c r="L12" s="3">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="M12" s="3">
+        <v>1.9E-3</v>
+      </c>
+      <c r="N12" s="3">
+        <v>0.1021</v>
+      </c>
+      <c r="O12" s="3">
+        <v>0</v>
       </c>
       <c r="P12">
         <v>2</v>
@@ -1897,17 +1555,17 @@
       <c r="Q12">
         <v>0</v>
       </c>
-      <c r="R12" t="s">
-        <v>29</v>
-      </c>
-      <c r="S12" t="s">
-        <v>24</v>
+      <c r="R12" s="3">
+        <v>6.1000000000000004E-3</v>
+      </c>
+      <c r="S12" s="3">
+        <v>0</v>
       </c>
       <c r="T12" s="1">
         <v>6777.9661016949158</v>
       </c>
-      <c r="U12" t="s">
-        <v>25</v>
+      <c r="U12" s="1">
+        <v>0</v>
       </c>
       <c r="V12">
         <v>1</v>
@@ -1918,49 +1576,49 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>196</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>197</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
-        <v>146</v>
-      </c>
-      <c r="F13" t="s">
-        <v>105</v>
+        <v>38</v>
+      </c>
+      <c r="F13" s="2">
+        <v>585</v>
       </c>
       <c r="G13">
         <v>15</v>
       </c>
-      <c r="H13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
-      <c r="J13" t="s">
-        <v>147</v>
+      <c r="H13" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="I13" s="3">
+        <v>6.7000000000000002E-3</v>
+      </c>
+      <c r="J13" s="2">
+        <v>862</v>
       </c>
       <c r="K13">
         <v>21</v>
       </c>
-      <c r="L13" t="s">
-        <v>73</v>
-      </c>
-      <c r="M13" t="s">
-        <v>81</v>
-      </c>
-      <c r="N13" t="s">
-        <v>148</v>
-      </c>
-      <c r="O13" t="s">
-        <v>38</v>
+      <c r="L13" s="3">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="M13" s="3">
+        <v>6.7999999999999996E-3</v>
+      </c>
+      <c r="N13" s="3">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="O13" s="3">
+        <v>8.3299999999999999E-2</v>
       </c>
       <c r="P13">
         <v>1</v>
@@ -1968,17 +1626,17 @@
       <c r="Q13">
         <v>0</v>
       </c>
-      <c r="R13" t="s">
-        <v>44</v>
-      </c>
-      <c r="S13" t="s">
-        <v>24</v>
+      <c r="R13" s="3">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="S13" s="3">
+        <v>0</v>
       </c>
       <c r="T13" s="1">
         <v>2117.7966101694915</v>
       </c>
-      <c r="U13" t="s">
-        <v>25</v>
+      <c r="U13" s="1">
+        <v>0</v>
       </c>
       <c r="V13">
         <v>1</v>
@@ -1989,49 +1647,49 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>180</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>102</v>
-      </c>
-      <c r="F14" t="s">
-        <v>103</v>
+        <v>22</v>
+      </c>
+      <c r="F14" s="2">
+        <v>446</v>
       </c>
       <c r="G14">
         <v>10</v>
       </c>
-      <c r="H14" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" t="s">
-        <v>104</v>
+      <c r="H14" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="I14" s="3">
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="J14" s="2">
+        <v>589</v>
       </c>
       <c r="K14">
         <v>13</v>
       </c>
-      <c r="L14" t="s">
-        <v>26</v>
-      </c>
-      <c r="M14" t="s">
-        <v>84</v>
-      </c>
-      <c r="N14" t="s">
-        <v>124</v>
-      </c>
-      <c r="O14" t="s">
-        <v>24</v>
+      <c r="L14" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="M14" s="3">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="N14" s="3">
+        <v>5.3900000000000003E-2</v>
+      </c>
+      <c r="O14" s="3">
+        <v>0</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -2039,17 +1697,17 @@
       <c r="Q14">
         <v>0</v>
       </c>
-      <c r="R14" t="s">
-        <v>24</v>
-      </c>
-      <c r="S14" t="s">
-        <v>24</v>
+      <c r="R14" s="3">
+        <v>0</v>
+      </c>
+      <c r="S14" s="3">
+        <v>0</v>
       </c>
       <c r="T14" s="1">
         <v>0</v>
       </c>
-      <c r="U14" t="s">
-        <v>25</v>
+      <c r="U14" s="1">
+        <v>0</v>
       </c>
       <c r="V14">
         <v>0</v>
@@ -2060,49 +1718,49 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s">
-        <v>199</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>150</v>
-      </c>
-      <c r="F15" t="s">
-        <v>78</v>
+        <v>40</v>
+      </c>
+      <c r="F15" s="2">
+        <v>140</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
-      <c r="H15" t="s">
-        <v>34</v>
-      </c>
-      <c r="I15" t="s">
-        <v>39</v>
-      </c>
-      <c r="J15" t="s">
-        <v>70</v>
+      <c r="H15" s="3">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="I15" s="3">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="J15" s="2">
+        <v>201</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
-      <c r="L15" t="s">
-        <v>35</v>
-      </c>
-      <c r="M15" t="s">
-        <v>58</v>
-      </c>
-      <c r="N15" t="s">
-        <v>151</v>
-      </c>
-      <c r="O15" t="s">
-        <v>24</v>
+      <c r="L15" s="3">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="M15" s="3">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="N15" s="3">
+        <v>8.7400000000000005E-2</v>
+      </c>
+      <c r="O15" s="3">
+        <v>0</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2110,17 +1768,17 @@
       <c r="Q15">
         <v>0</v>
       </c>
-      <c r="R15" t="s">
-        <v>24</v>
-      </c>
-      <c r="S15" t="s">
-        <v>24</v>
+      <c r="R15" s="3">
+        <v>0</v>
+      </c>
+      <c r="S15" s="3">
+        <v>0</v>
       </c>
       <c r="T15" s="1">
         <v>0</v>
       </c>
-      <c r="U15" t="s">
-        <v>25</v>
+      <c r="U15" s="1">
+        <v>0</v>
       </c>
       <c r="V15">
         <v>0</v>
@@ -2131,49 +1789,49 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
-        <v>201</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>152</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>152</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
-        <v>153</v>
-      </c>
-      <c r="F16" t="s">
-        <v>98</v>
+        <v>42</v>
+      </c>
+      <c r="F16" s="2">
+        <v>26</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
-      <c r="H16" t="s">
-        <v>57</v>
-      </c>
-      <c r="I16" t="s">
-        <v>24</v>
-      </c>
-      <c r="J16" t="s">
-        <v>113</v>
+      <c r="H16" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="I16" s="3">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>39</v>
       </c>
       <c r="K16">
         <v>0</v>
       </c>
-      <c r="L16" t="s">
-        <v>57</v>
-      </c>
-      <c r="M16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N16" t="s">
-        <v>23</v>
-      </c>
-      <c r="O16" t="s">
-        <v>24</v>
+      <c r="L16" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="M16" s="3">
+        <v>0</v>
+      </c>
+      <c r="N16" s="3">
+        <v>1</v>
+      </c>
+      <c r="O16" s="3">
+        <v>0</v>
       </c>
       <c r="P16">
         <v>0</v>
@@ -2181,17 +1839,17 @@
       <c r="Q16">
         <v>0</v>
       </c>
-      <c r="R16" t="s">
-        <v>24</v>
-      </c>
-      <c r="S16" t="s">
-        <v>24</v>
+      <c r="R16" s="3">
+        <v>0</v>
+      </c>
+      <c r="S16" s="3">
+        <v>0</v>
       </c>
       <c r="T16" s="1">
         <v>0</v>
       </c>
-      <c r="U16" t="s">
-        <v>25</v>
+      <c r="U16" s="1">
+        <v>0</v>
       </c>
       <c r="V16">
         <v>0</v>
@@ -2202,49 +1860,49 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>202</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>203</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>43</v>
       </c>
       <c r="D17" t="s">
-        <v>154</v>
+        <v>43</v>
       </c>
       <c r="E17" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" t="s">
-        <v>114</v>
+        <v>44</v>
+      </c>
+      <c r="F17" s="2">
+        <v>17</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" t="s">
-        <v>24</v>
-      </c>
-      <c r="J17" t="s">
-        <v>56</v>
+      <c r="H17" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>20</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
-      <c r="L17" t="s">
-        <v>41</v>
-      </c>
-      <c r="M17" t="s">
-        <v>24</v>
-      </c>
-      <c r="N17" t="s">
-        <v>24</v>
-      </c>
-      <c r="O17" t="s">
-        <v>24</v>
+      <c r="L17" s="3">
+        <v>1E-4</v>
+      </c>
+      <c r="M17" s="3">
+        <v>0</v>
+      </c>
+      <c r="N17" s="3">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3">
+        <v>0</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -2252,17 +1910,17 @@
       <c r="Q17">
         <v>0</v>
       </c>
-      <c r="R17" t="s">
-        <v>24</v>
-      </c>
-      <c r="S17" t="s">
-        <v>24</v>
+      <c r="R17" s="3">
+        <v>0</v>
+      </c>
+      <c r="S17" s="3">
+        <v>0</v>
       </c>
       <c r="T17" s="1">
         <v>0</v>
       </c>
-      <c r="U17" t="s">
-        <v>25</v>
+      <c r="U17" s="1">
+        <v>0</v>
       </c>
       <c r="V17">
         <v>0</v>
@@ -2273,49 +1931,49 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>204</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>205</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>157</v>
-      </c>
-      <c r="F18" t="s">
-        <v>100</v>
+        <v>46</v>
+      </c>
+      <c r="F18" s="2">
+        <v>27</v>
       </c>
       <c r="G18">
         <v>2</v>
       </c>
-      <c r="H18" t="s">
-        <v>57</v>
-      </c>
-      <c r="I18" t="s">
-        <v>62</v>
-      </c>
-      <c r="J18" t="s">
-        <v>92</v>
+      <c r="H18" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="I18" s="3">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="J18" s="2">
+        <v>37</v>
       </c>
       <c r="K18">
         <v>2</v>
       </c>
-      <c r="L18" t="s">
-        <v>57</v>
-      </c>
-      <c r="M18" t="s">
-        <v>40</v>
-      </c>
-      <c r="N18" t="s">
-        <v>85</v>
-      </c>
-      <c r="O18" t="s">
-        <v>24</v>
+      <c r="L18" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="M18" s="3">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="N18" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="O18" s="3">
+        <v>0</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -2323,17 +1981,17 @@
       <c r="Q18">
         <v>0</v>
       </c>
-      <c r="R18" t="s">
-        <v>24</v>
-      </c>
-      <c r="S18" t="s">
-        <v>24</v>
+      <c r="R18" s="3">
+        <v>0</v>
+      </c>
+      <c r="S18" s="3">
+        <v>0</v>
       </c>
       <c r="T18" s="1">
         <v>0</v>
       </c>
-      <c r="U18" t="s">
-        <v>25</v>
+      <c r="U18" s="1">
+        <v>0</v>
       </c>
       <c r="V18">
         <v>0</v>
@@ -2344,49 +2002,49 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>206</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>158</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>158</v>
+        <v>47</v>
       </c>
       <c r="E19" t="s">
-        <v>159</v>
-      </c>
-      <c r="F19" t="s">
-        <v>160</v>
+        <v>48</v>
+      </c>
+      <c r="F19" s="2">
+        <v>18</v>
       </c>
       <c r="G19">
         <v>0</v>
       </c>
-      <c r="H19" t="s">
-        <v>57</v>
-      </c>
-      <c r="I19" t="s">
-        <v>24</v>
-      </c>
-      <c r="J19" t="s">
-        <v>99</v>
+      <c r="H19" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="I19" s="3">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2">
+        <v>32</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
-      <c r="L19" t="s">
-        <v>57</v>
-      </c>
-      <c r="M19" t="s">
-        <v>24</v>
-      </c>
-      <c r="N19" t="s">
-        <v>23</v>
-      </c>
-      <c r="O19" t="s">
-        <v>24</v>
+      <c r="L19" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="M19" s="3">
+        <v>0</v>
+      </c>
+      <c r="N19" s="3">
+        <v>1</v>
+      </c>
+      <c r="O19" s="3">
+        <v>0</v>
       </c>
       <c r="P19">
         <v>0</v>
@@ -2394,17 +2052,17 @@
       <c r="Q19">
         <v>0</v>
       </c>
-      <c r="R19" t="s">
-        <v>24</v>
-      </c>
-      <c r="S19" t="s">
-        <v>24</v>
+      <c r="R19" s="3">
+        <v>0</v>
+      </c>
+      <c r="S19" s="3">
+        <v>0</v>
       </c>
       <c r="T19" s="1">
         <v>0</v>
       </c>
-      <c r="U19" t="s">
-        <v>25</v>
+      <c r="U19" s="1">
+        <v>0</v>
       </c>
       <c r="V19">
         <v>0</v>
@@ -2415,49 +2073,49 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>208</v>
+        <v>93</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="D20" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
-        <v>162</v>
-      </c>
-      <c r="F20" t="s">
-        <v>98</v>
+        <v>50</v>
+      </c>
+      <c r="F20" s="2">
+        <v>26</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
-      <c r="H20" t="s">
-        <v>57</v>
-      </c>
-      <c r="I20" t="s">
-        <v>24</v>
-      </c>
-      <c r="J20" t="s">
-        <v>115</v>
+      <c r="H20" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="I20" s="3">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>30</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
-      <c r="L20" t="s">
-        <v>57</v>
-      </c>
-      <c r="M20" t="s">
-        <v>24</v>
-      </c>
-      <c r="N20" t="s">
-        <v>76</v>
-      </c>
-      <c r="O20" t="s">
-        <v>24</v>
+      <c r="L20" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="M20" s="3">
+        <v>0</v>
+      </c>
+      <c r="N20" s="3">
+        <v>0.1111</v>
+      </c>
+      <c r="O20" s="3">
+        <v>0</v>
       </c>
       <c r="P20">
         <v>0</v>
@@ -2465,17 +2123,17 @@
       <c r="Q20">
         <v>0</v>
       </c>
-      <c r="R20" t="s">
-        <v>24</v>
-      </c>
-      <c r="S20" t="s">
-        <v>24</v>
+      <c r="R20" s="3">
+        <v>0</v>
+      </c>
+      <c r="S20" s="3">
+        <v>0</v>
       </c>
       <c r="T20" s="1">
         <v>0</v>
       </c>
-      <c r="U20" t="s">
-        <v>25</v>
+      <c r="U20" s="1">
+        <v>0</v>
       </c>
       <c r="V20">
         <v>0</v>
@@ -2486,49 +2144,49 @@
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>210</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>211</v>
+        <v>96</v>
       </c>
       <c r="C21" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="E21" t="s">
-        <v>164</v>
-      </c>
-      <c r="F21" t="s">
-        <v>165</v>
+        <v>52</v>
+      </c>
+      <c r="F21" s="2">
+        <v>626</v>
       </c>
       <c r="G21">
         <v>6</v>
       </c>
-      <c r="H21" t="s">
-        <v>82</v>
-      </c>
-      <c r="I21" t="s">
-        <v>61</v>
-      </c>
-      <c r="J21" t="s">
-        <v>166</v>
+      <c r="H21" s="3">
+        <v>5.4000000000000003E-3</v>
+      </c>
+      <c r="I21" s="3">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="J21" s="2">
+        <v>817</v>
       </c>
       <c r="K21">
         <v>6</v>
       </c>
-      <c r="L21" t="s">
-        <v>27</v>
-      </c>
-      <c r="M21" t="s">
-        <v>47</v>
-      </c>
-      <c r="N21" t="s">
-        <v>59</v>
-      </c>
-      <c r="O21" t="s">
-        <v>24</v>
+      <c r="L21" s="3">
+        <v>5.1999999999999998E-3</v>
+      </c>
+      <c r="M21" s="3">
+        <v>1.9E-3</v>
+      </c>
+      <c r="N21" s="3">
+        <v>2.92E-2</v>
+      </c>
+      <c r="O21" s="3">
+        <v>0</v>
       </c>
       <c r="P21">
         <v>0</v>
@@ -2536,17 +2194,17 @@
       <c r="Q21">
         <v>0</v>
       </c>
-      <c r="R21" t="s">
-        <v>24</v>
-      </c>
-      <c r="S21" t="s">
-        <v>24</v>
+      <c r="R21" s="3">
+        <v>0</v>
+      </c>
+      <c r="S21" s="3">
+        <v>0</v>
       </c>
       <c r="T21" s="1">
         <v>0</v>
       </c>
-      <c r="U21" t="s">
-        <v>25</v>
+      <c r="U21" s="1">
+        <v>0</v>
       </c>
       <c r="V21">
         <v>0</v>
@@ -2557,49 +2215,49 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>212</v>
+        <v>97</v>
       </c>
       <c r="B22" t="s">
-        <v>213</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="E22" t="s">
-        <v>168</v>
-      </c>
-      <c r="F22" t="s">
-        <v>79</v>
+        <v>54</v>
+      </c>
+      <c r="F22" s="2">
+        <v>4</v>
       </c>
       <c r="G22">
         <v>0</v>
       </c>
-      <c r="H22" t="s">
-        <v>24</v>
-      </c>
-      <c r="I22" t="s">
-        <v>24</v>
-      </c>
-      <c r="J22" t="s">
-        <v>65</v>
+      <c r="H22" s="3">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2">
+        <v>5</v>
       </c>
       <c r="K22">
         <v>0</v>
       </c>
-      <c r="L22" t="s">
-        <v>24</v>
-      </c>
-      <c r="M22" t="s">
-        <v>24</v>
-      </c>
-      <c r="N22" t="s">
-        <v>23</v>
-      </c>
-      <c r="O22" t="s">
-        <v>24</v>
+      <c r="L22" s="3">
+        <v>0</v>
+      </c>
+      <c r="M22" s="3">
+        <v>0</v>
+      </c>
+      <c r="N22" s="3">
+        <v>1</v>
+      </c>
+      <c r="O22" s="3">
+        <v>0</v>
       </c>
       <c r="P22">
         <v>0</v>
@@ -2607,17 +2265,17 @@
       <c r="Q22">
         <v>0</v>
       </c>
-      <c r="R22" t="s">
-        <v>24</v>
-      </c>
-      <c r="S22" t="s">
-        <v>24</v>
+      <c r="R22" s="3">
+        <v>0</v>
+      </c>
+      <c r="S22" s="3">
+        <v>0</v>
       </c>
       <c r="T22" s="1">
         <v>0</v>
       </c>
-      <c r="U22" t="s">
-        <v>25</v>
+      <c r="U22" s="1">
+        <v>0</v>
       </c>
       <c r="V22">
         <v>0</v>
@@ -2628,49 +2286,49 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>214</v>
+        <v>99</v>
       </c>
       <c r="B23" t="s">
-        <v>215</v>
+        <v>100</v>
       </c>
       <c r="C23" t="s">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="E23" t="s">
-        <v>170</v>
-      </c>
-      <c r="F23" t="s">
-        <v>97</v>
+        <v>56</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
       </c>
       <c r="G23">
         <v>0</v>
       </c>
-      <c r="H23" t="s">
-        <v>24</v>
-      </c>
-      <c r="I23" t="s">
-        <v>24</v>
-      </c>
-      <c r="J23" t="s">
-        <v>97</v>
+      <c r="H23" s="3">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2">
+        <v>0</v>
       </c>
       <c r="K23">
         <v>0</v>
       </c>
-      <c r="L23" t="s">
-        <v>24</v>
-      </c>
-      <c r="M23" t="s">
-        <v>24</v>
-      </c>
-      <c r="N23" t="s">
-        <v>24</v>
-      </c>
-      <c r="O23" t="s">
-        <v>24</v>
+      <c r="L23" s="3">
+        <v>0</v>
+      </c>
+      <c r="M23" s="3">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3">
+        <v>0</v>
+      </c>
+      <c r="O23" s="3">
+        <v>0</v>
       </c>
       <c r="P23">
         <v>0</v>
@@ -2678,17 +2336,17 @@
       <c r="Q23">
         <v>0</v>
       </c>
-      <c r="R23" t="s">
-        <v>24</v>
-      </c>
-      <c r="S23" t="s">
-        <v>24</v>
+      <c r="R23" s="3">
+        <v>0</v>
+      </c>
+      <c r="S23" s="3">
+        <v>0</v>
       </c>
       <c r="T23" s="1">
         <v>0</v>
       </c>
-      <c r="U23" t="s">
-        <v>25</v>
+      <c r="U23" s="1">
+        <v>0</v>
       </c>
       <c r="V23">
         <v>0</v>
@@ -2699,49 +2357,49 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>216</v>
+        <v>101</v>
       </c>
       <c r="B24" t="s">
-        <v>217</v>
+        <v>102</v>
       </c>
       <c r="C24" t="s">
-        <v>171</v>
+        <v>57</v>
       </c>
       <c r="D24" t="s">
-        <v>171</v>
+        <v>57</v>
       </c>
       <c r="E24" t="s">
-        <v>172</v>
-      </c>
-      <c r="F24" t="s">
-        <v>95</v>
+        <v>58</v>
+      </c>
+      <c r="F24" s="2">
+        <v>178</v>
       </c>
       <c r="G24">
         <v>10</v>
       </c>
-      <c r="H24" t="s">
-        <v>53</v>
-      </c>
-      <c r="I24" t="s">
-        <v>48</v>
-      </c>
-      <c r="J24" t="s">
-        <v>173</v>
+      <c r="H24" s="3">
+        <v>1.5E-3</v>
+      </c>
+      <c r="I24" s="3">
+        <v>4.4000000000000003E-3</v>
+      </c>
+      <c r="J24" s="2">
+        <v>211</v>
       </c>
       <c r="K24">
         <v>10</v>
       </c>
-      <c r="L24" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" t="s">
-        <v>43</v>
-      </c>
-      <c r="N24" t="s">
-        <v>24</v>
-      </c>
-      <c r="O24" t="s">
-        <v>24</v>
+      <c r="L24" s="3">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="M24" s="3">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="N24" s="3">
+        <v>0</v>
+      </c>
+      <c r="O24" s="3">
+        <v>0</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -2749,17 +2407,17 @@
       <c r="Q24">
         <v>0</v>
       </c>
-      <c r="R24" t="s">
-        <v>24</v>
-      </c>
-      <c r="S24" t="s">
-        <v>24</v>
+      <c r="R24" s="3">
+        <v>0</v>
+      </c>
+      <c r="S24" s="3">
+        <v>0</v>
       </c>
       <c r="T24" s="1">
         <v>0</v>
       </c>
-      <c r="U24" t="s">
-        <v>25</v>
+      <c r="U24" s="1">
+        <v>0</v>
       </c>
       <c r="V24">
         <v>0</v>
@@ -2770,16 +2428,16 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>186</v>
+        <v>71</v>
       </c>
       <c r="B25" t="s">
-        <v>187</v>
+        <v>72</v>
       </c>
       <c r="C25" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>125</v>
+        <v>27</v>
       </c>
       <c r="P25">
         <v>27</v>
@@ -2790,16 +2448,16 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>214</v>
+        <v>99</v>
       </c>
       <c r="B26" t="s">
-        <v>215</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="D26" t="s">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="P26">
         <v>18</v>
@@ -2810,16 +2468,16 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>196</v>
+        <v>81</v>
       </c>
       <c r="B27" t="s">
-        <v>197</v>
+        <v>82</v>
       </c>
       <c r="C27" t="s">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="D27" t="s">
-        <v>145</v>
+        <v>37</v>
       </c>
       <c r="P27">
         <v>8</v>
@@ -2830,16 +2488,16 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>178</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>179</v>
+        <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="P28">
         <v>8</v>
@@ -2850,16 +2508,16 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>190</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
-        <v>191</v>
+        <v>76</v>
       </c>
       <c r="C29" t="s">
-        <v>134</v>
+        <v>31</v>
       </c>
       <c r="D29" t="s">
-        <v>134</v>
+        <v>31</v>
       </c>
       <c r="P29">
         <v>6</v>
@@ -2870,16 +2528,16 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="B30" t="s">
-        <v>199</v>
+        <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="D30" t="s">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="P30">
         <v>6</v>
@@ -2890,16 +2548,16 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>180</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s">
-        <v>181</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="P31">
         <v>6</v>
@@ -2910,16 +2568,16 @@
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>218</v>
+        <v>103</v>
       </c>
       <c r="B32" t="s">
-        <v>219</v>
+        <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>220</v>
+        <v>105</v>
       </c>
       <c r="D32" t="s">
-        <v>220</v>
+        <v>105</v>
       </c>
       <c r="P32">
         <v>7</v>
@@ -2930,16 +2588,16 @@
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>194</v>
+        <v>79</v>
       </c>
       <c r="B33" t="s">
-        <v>195</v>
+        <v>80</v>
       </c>
       <c r="C33" t="s">
-        <v>141</v>
+        <v>35</v>
       </c>
       <c r="D33" t="s">
-        <v>141</v>
+        <v>35</v>
       </c>
       <c r="P33">
         <v>3</v>
@@ -2950,16 +2608,16 @@
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>221</v>
+        <v>106</v>
       </c>
       <c r="B34" t="s">
-        <v>222</v>
+        <v>107</v>
       </c>
       <c r="C34" t="s">
-        <v>223</v>
+        <v>108</v>
       </c>
       <c r="D34" t="s">
-        <v>223</v>
+        <v>108</v>
       </c>
       <c r="P34">
         <v>2</v>
@@ -2970,16 +2628,16 @@
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>182</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>183</v>
+        <v>68</v>
       </c>
       <c r="C35" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="D35" t="s">
-        <v>108</v>
+        <v>23</v>
       </c>
       <c r="P35">
         <v>2</v>
@@ -2990,16 +2648,16 @@
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>188</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>189</v>
+        <v>74</v>
       </c>
       <c r="C36" t="s">
-        <v>129</v>
+        <v>29</v>
       </c>
       <c r="D36" t="s">
-        <v>129</v>
+        <v>29</v>
       </c>
       <c r="P36">
         <v>4</v>
@@ -3010,16 +2668,16 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>224</v>
+        <v>109</v>
       </c>
       <c r="B37" t="s">
-        <v>225</v>
+        <v>110</v>
       </c>
       <c r="C37" t="s">
-        <v>226</v>
+        <v>111</v>
       </c>
       <c r="D37" t="s">
-        <v>226</v>
+        <v>111</v>
       </c>
       <c r="P37">
         <v>1</v>
@@ -3030,16 +2688,16 @@
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>210</v>
+        <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>211</v>
+        <v>96</v>
       </c>
       <c r="C38" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="D38" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="P38">
         <v>1</v>
@@ -3050,16 +2708,16 @@
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>192</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>193</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="D39" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="P39">
         <v>1</v>

</xml_diff>